<commit_message>
Add zodiac, letter, and number spacers plus refreshed bead hero images.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/new_input/commodity_idx.xlsx
+++ b/new_input/commodity_idx.xlsx
@@ -432,7 +432,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -487,12 +487,36 @@
         <v>配件</v>
       </c>
       <c r="B7" t="str">
+        <v>字母</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>配件</v>
+      </c>
+      <c r="B8" t="str">
+        <v>數字</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>配件</v>
+      </c>
+      <c r="B9" t="str">
+        <v>星座</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>配件</v>
+      </c>
+      <c r="B10" t="str">
         <v>隔珠</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add accessory high_mm/supply fields and refresh catalog from xlsx.
Accessories now store cord size vs face height; accessory-only sync replaces the full accessory set, and DIY layout uses highMm for pendant bodies and charm faces.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/new_input/commodity_idx.xlsx
+++ b/new_input/commodity_idx.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,15 +417,21 @@
         <v>size_mm</v>
       </c>
       <c r="F1" t="str">
+        <v>high_mm</v>
+      </c>
+      <c r="G1" t="str">
         <v>price_twd</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>picture</v>
+      </c>
+      <c r="I1" t="str">
+        <v>supply</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>